<commit_message>
Add round forecast to whole units and update results
</commit_message>
<xml_diff>
--- a/outputs/Erratic/Erratic - High N_d_report.xlsx
+++ b/outputs/Erratic/Erratic - High N_d_report.xlsx
@@ -511,13 +511,13 @@
         <v>40</v>
       </c>
       <c r="D4" t="n">
-        <v>1.667052414977889</v>
+        <v>1.671126414370071</v>
       </c>
       <c r="E4" t="n">
-        <v>1.508575457495892</v>
+        <v>1.507691182527639</v>
       </c>
       <c r="F4" t="n">
-        <v>130</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5">
@@ -532,16 +532,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>25.00000074505805</v>
+        <v>25</v>
       </c>
       <c r="D5" t="n">
-        <v>1.720291143937981</v>
+        <v>1.718688405861801</v>
       </c>
       <c r="E5" t="n">
-        <v>1.507697406961698</v>
+        <v>1.509140927361087</v>
       </c>
       <c r="F5" t="n">
-        <v>227.3757068596256</v>
+        <v>230</v>
       </c>
     </row>
     <row r="6">
@@ -556,16 +556,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>25.58947735595949</v>
+        <v>26</v>
       </c>
       <c r="D6" t="n">
-        <v>1.769920351271141</v>
+        <v>1.77128892238078</v>
       </c>
       <c r="E6" t="n">
-        <v>1.531236098482712</v>
+        <v>1.532343087833938</v>
       </c>
       <c r="F6" t="n">
-        <v>17.41669725461996</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -580,16 +580,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>62.91640248069407</v>
+        <v>63</v>
       </c>
       <c r="D7" t="n">
-        <v>1.945193970874192</v>
+        <v>1.945578478609262</v>
       </c>
       <c r="E7" t="n">
-        <v>1.795979560844699</v>
+        <v>1.795537875282427</v>
       </c>
       <c r="F7" t="n">
-        <v>733.0956679742322</v>
+        <v>730</v>
       </c>
     </row>
     <row r="8">
@@ -604,16 +604,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>56.62476223262466</v>
+        <v>57</v>
       </c>
       <c r="D8" t="n">
-        <v>1.95944468527349</v>
+        <v>1.949855853153142</v>
       </c>
       <c r="E8" t="n">
-        <v>1.82736031331668</v>
+        <v>1.825820662856621</v>
       </c>
       <c r="F8" t="n">
-        <v>829.786101176809</v>
+        <v>834</v>
       </c>
     </row>
     <row r="9">
@@ -628,16 +628,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>68.15635078589283</v>
+        <v>68</v>
       </c>
       <c r="D9" t="n">
-        <v>1.927882160592601</v>
+        <v>1.928598540824044</v>
       </c>
       <c r="E9" t="n">
-        <v>1.665661894932681</v>
+        <v>1.665167672625313</v>
       </c>
       <c r="F9" t="n">
-        <v>353.5564386807393</v>
+        <v>353</v>
       </c>
     </row>
     <row r="10">
@@ -700,16 +700,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>227.5</v>
+        <v>228</v>
       </c>
       <c r="D12" t="n">
-        <v>2.19066590922729</v>
+        <v>2.194131218427894</v>
       </c>
       <c r="E12" t="n">
-        <v>2.390094885337331</v>
+        <v>2.390315999710049</v>
       </c>
       <c r="F12" t="n">
-        <v>222.5</v>
+        <v>220</v>
       </c>
     </row>
     <row r="13">
@@ -724,16 +724,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>243.4562003271037</v>
+        <v>243</v>
       </c>
       <c r="D13" t="n">
-        <v>2.76370886924275</v>
+        <v>2.766297456938122</v>
       </c>
       <c r="E13" t="n">
-        <v>2.621736657331293</v>
+        <v>2.623139611266071</v>
       </c>
       <c r="F13" t="n">
-        <v>228.4212215883764</v>
+        <v>228</v>
       </c>
     </row>
     <row r="14">
@@ -748,16 +748,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>276.8749091902814</v>
+        <v>277</v>
       </c>
       <c r="D14" t="n">
-        <v>3.03153636293224</v>
+        <v>3.032679912152875</v>
       </c>
       <c r="E14" t="n">
-        <v>2.72034450036592</v>
+        <v>2.721130056160801</v>
       </c>
       <c r="F14" t="n">
-        <v>-148.1469737592385</v>
+        <v>-148</v>
       </c>
     </row>
     <row r="15">
@@ -772,16 +772,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>118.3583574964666</v>
+        <v>118</v>
       </c>
       <c r="D15" t="n">
-        <v>2.617974675556236</v>
+        <v>2.616739573737839</v>
       </c>
       <c r="E15" t="n">
-        <v>2.791646141495675</v>
+        <v>2.793243061210935</v>
       </c>
       <c r="F15" t="n">
-        <v>1191.642120703956</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="16">
@@ -796,16 +796,16 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>106.52252174682</v>
+        <v>107</v>
       </c>
       <c r="D16" t="n">
-        <v>2.658307148108265</v>
+        <v>2.65500552394871</v>
       </c>
       <c r="E16" t="n">
-        <v>2.820362305142265</v>
+        <v>2.817281807502502</v>
       </c>
       <c r="F16" t="n">
-        <v>1242.47790863356</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="17">
@@ -820,16 +820,16 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>161.7224922862985</v>
+        <v>162</v>
       </c>
       <c r="D17" t="n">
-        <v>2.497218739829018</v>
+        <v>2.499005642327436</v>
       </c>
       <c r="E17" t="n">
-        <v>2.637843492555762</v>
+        <v>2.637465406086856</v>
       </c>
       <c r="F17" t="n">
-        <v>936.749937604086</v>
+        <v>937</v>
       </c>
     </row>
     <row r="18">
@@ -892,16 +892,16 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>717.5</v>
+        <v>718</v>
       </c>
       <c r="D20" t="n">
-        <v>1.138636363636364</v>
+        <v>1.14</v>
       </c>
       <c r="E20" t="n">
-        <v>0.738523669159449</v>
+        <v>0.7394081286434723</v>
       </c>
       <c r="F20" t="n">
-        <v>-417.5</v>
+        <v>-418</v>
       </c>
     </row>
     <row r="21">
@@ -916,16 +916,16 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1124.999985471368</v>
+        <v>1125</v>
       </c>
       <c r="D21" t="n">
-        <v>6.338888810437621</v>
+        <v>6.336666666666666</v>
       </c>
       <c r="E21" t="n">
-        <v>8.897393571812778</v>
+        <v>8.897103015513858</v>
       </c>
       <c r="F21" t="n">
-        <v>237.4999996998508</v>
+        <v>237</v>
       </c>
     </row>
     <row r="22">
@@ -940,16 +940,16 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1187.501874203842</v>
+        <v>1188</v>
       </c>
       <c r="D22" t="n">
-        <v>5.762375454085102</v>
+        <v>5.761050505050505</v>
       </c>
       <c r="E22" t="n">
-        <v>8.279890793350983</v>
+        <v>8.27694606529786</v>
       </c>
       <c r="F22" t="n">
-        <v>-4.16853838965153</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="23">
@@ -964,16 +964,16 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>274.6</v>
+        <v>275</v>
       </c>
       <c r="D23" t="n">
-        <v>6.181313131313131</v>
+        <v>6.180949494949494</v>
       </c>
       <c r="E23" t="n">
-        <v>9.666080647454995</v>
+        <v>9.666079559765922</v>
       </c>
       <c r="F23" t="n">
-        <v>1273.4</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="24">
@@ -988,16 +988,16 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>247.14</v>
+        <v>247</v>
       </c>
       <c r="D24" t="n">
-        <v>6.257121212121213</v>
+        <v>6.256181818181818</v>
       </c>
       <c r="E24" t="n">
-        <v>9.724872300978284</v>
+        <v>9.723068873463902</v>
       </c>
       <c r="F24" t="n">
-        <v>1313.56</v>
+        <v>1313</v>
       </c>
     </row>
     <row r="25">
@@ -1012,16 +1012,16 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>274.6</v>
+        <v>275</v>
       </c>
       <c r="D25" t="n">
-        <v>6.181313131313131</v>
+        <v>6.180949494949494</v>
       </c>
       <c r="E25" t="n">
-        <v>9.666080647454995</v>
+        <v>9.666079559765922</v>
       </c>
       <c r="F25" t="n">
-        <v>1273.4</v>
+        <v>1273</v>
       </c>
     </row>
   </sheetData>

</xml_diff>